<commit_message>
Auto update PropHit model output and snapshots
</commit_message>
<xml_diff>
--- a/outputs/prophit_today.xlsx
+++ b/outputs/prophit_today.xlsx
@@ -2177,7 +2177,7 @@
       </c>
       <c r="HB2" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC2" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="HE2" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c r="HB3" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC3" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="HE3" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="HB4" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC4" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="HE4" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="HB5" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC5" t="inlineStr">
@@ -4323,7 +4323,7 @@
       </c>
       <c r="HE5" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="HB6" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC6" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="HE6" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
       </c>
       <c r="HB7" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC7" t="inlineStr">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="HE7" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="HB8" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC8" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="HE8" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -7154,7 +7154,7 @@
       </c>
       <c r="HB9" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC9" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="HE9" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="HB10" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC10" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="HE10" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -8576,7 +8576,7 @@
       </c>
       <c r="HB11" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC11" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="HE11" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -9287,7 +9287,7 @@
       </c>
       <c r="HB12" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC12" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="HE12" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -9998,7 +9998,7 @@
       </c>
       <c r="HB13" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC13" t="inlineStr">
@@ -10011,7 +10011,7 @@
       </c>
       <c r="HE13" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -10709,7 +10709,7 @@
       </c>
       <c r="HB14" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC14" t="inlineStr">
@@ -10722,7 +10722,7 @@
       </c>
       <c r="HE14" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -11420,7 +11420,7 @@
       </c>
       <c r="HB15" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC15" t="inlineStr">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="HE15" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="HB16" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC16" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="HE16" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -12842,7 +12842,7 @@
       </c>
       <c r="HB17" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC17" t="inlineStr">
@@ -12855,7 +12855,7 @@
       </c>
       <c r="HE17" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -13553,7 +13553,7 @@
       </c>
       <c r="HB18" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC18" t="inlineStr">
@@ -13566,7 +13566,7 @@
       </c>
       <c r="HE18" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -14264,7 +14264,7 @@
       </c>
       <c r="HB19" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC19" t="inlineStr">
@@ -14277,7 +14277,7 @@
       </c>
       <c r="HE19" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -14975,7 +14975,7 @@
       </c>
       <c r="HB20" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC20" t="inlineStr">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="HE20" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -15686,7 +15686,7 @@
       </c>
       <c r="HB21" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC21" t="inlineStr">
@@ -15699,7 +15699,7 @@
       </c>
       <c r="HE21" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -16397,7 +16397,7 @@
       </c>
       <c r="HB22" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC22" t="inlineStr">
@@ -16410,7 +16410,7 @@
       </c>
       <c r="HE22" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -17108,7 +17108,7 @@
       </c>
       <c r="HB23" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC23" t="inlineStr">
@@ -17121,7 +17121,7 @@
       </c>
       <c r="HE23" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -17819,7 +17819,7 @@
       </c>
       <c r="HB24" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC24" t="inlineStr">
@@ -17832,7 +17832,7 @@
       </c>
       <c r="HE24" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -18530,7 +18530,7 @@
       </c>
       <c r="HB25" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC25" t="inlineStr">
@@ -18543,7 +18543,7 @@
       </c>
       <c r="HE25" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -19241,7 +19241,7 @@
       </c>
       <c r="HB26" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC26" t="inlineStr">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="HE26" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -19952,7 +19952,7 @@
       </c>
       <c r="HB27" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC27" t="inlineStr">
@@ -19965,7 +19965,7 @@
       </c>
       <c r="HE27" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -20663,7 +20663,7 @@
       </c>
       <c r="HB28" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC28" t="inlineStr">
@@ -20676,7 +20676,7 @@
       </c>
       <c r="HE28" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="HB29" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC29" t="inlineStr">
@@ -21387,7 +21387,7 @@
       </c>
       <c r="HE29" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -22085,7 +22085,7 @@
       </c>
       <c r="HB30" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC30" t="inlineStr">
@@ -22098,7 +22098,7 @@
       </c>
       <c r="HE30" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -22796,7 +22796,7 @@
       </c>
       <c r="HB31" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC31" t="inlineStr">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="HE31" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -23507,7 +23507,7 @@
       </c>
       <c r="HB32" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC32" t="inlineStr">
@@ -23520,7 +23520,7 @@
       </c>
       <c r="HE32" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -24218,7 +24218,7 @@
       </c>
       <c r="HB33" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC33" t="inlineStr">
@@ -24231,7 +24231,7 @@
       </c>
       <c r="HE33" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -24929,7 +24929,7 @@
       </c>
       <c r="HB34" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC34" t="inlineStr">
@@ -24942,7 +24942,7 @@
       </c>
       <c r="HE34" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -25640,7 +25640,7 @@
       </c>
       <c r="HB35" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC35" t="inlineStr">
@@ -25653,7 +25653,7 @@
       </c>
       <c r="HE35" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -26351,7 +26351,7 @@
       </c>
       <c r="HB36" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC36" t="inlineStr">
@@ -26364,7 +26364,7 @@
       </c>
       <c r="HE36" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -27062,7 +27062,7 @@
       </c>
       <c r="HB37" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC37" t="inlineStr">
@@ -27075,7 +27075,7 @@
       </c>
       <c r="HE37" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -27773,7 +27773,7 @@
       </c>
       <c r="HB38" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC38" t="inlineStr">
@@ -27786,7 +27786,7 @@
       </c>
       <c r="HE38" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -28484,7 +28484,7 @@
       </c>
       <c r="HB39" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC39" t="inlineStr">
@@ -28497,7 +28497,7 @@
       </c>
       <c r="HE39" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -29191,7 +29191,7 @@
       </c>
       <c r="HB40" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC40" t="inlineStr">
@@ -29204,7 +29204,7 @@
       </c>
       <c r="HE40" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -29902,7 +29902,7 @@
       </c>
       <c r="HB41" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC41" t="inlineStr">
@@ -29915,7 +29915,7 @@
       </c>
       <c r="HE41" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -30613,7 +30613,7 @@
       </c>
       <c r="HB42" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC42" t="inlineStr">
@@ -30626,7 +30626,7 @@
       </c>
       <c r="HE42" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -31324,7 +31324,7 @@
       </c>
       <c r="HB43" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC43" t="inlineStr">
@@ -31337,7 +31337,7 @@
       </c>
       <c r="HE43" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -32035,7 +32035,7 @@
       </c>
       <c r="HB44" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC44" t="inlineStr">
@@ -32048,7 +32048,7 @@
       </c>
       <c r="HE44" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -32746,7 +32746,7 @@
       </c>
       <c r="HB45" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC45" t="inlineStr">
@@ -32759,7 +32759,7 @@
       </c>
       <c r="HE45" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -33457,7 +33457,7 @@
       </c>
       <c r="HB46" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC46" t="inlineStr">
@@ -33470,7 +33470,7 @@
       </c>
       <c r="HE46" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -34168,7 +34168,7 @@
       </c>
       <c r="HB47" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC47" t="inlineStr">
@@ -34181,7 +34181,7 @@
       </c>
       <c r="HE47" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -34879,7 +34879,7 @@
       </c>
       <c r="HB48" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC48" t="inlineStr">
@@ -34892,7 +34892,7 @@
       </c>
       <c r="HE48" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -35590,7 +35590,7 @@
       </c>
       <c r="HB49" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC49" t="inlineStr">
@@ -35603,7 +35603,7 @@
       </c>
       <c r="HE49" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -36297,7 +36297,7 @@
       </c>
       <c r="HB50" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC50" t="inlineStr">
@@ -36310,7 +36310,7 @@
       </c>
       <c r="HE50" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -37008,7 +37008,7 @@
       </c>
       <c r="HB51" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC51" t="inlineStr">
@@ -37021,7 +37021,7 @@
       </c>
       <c r="HE51" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -37719,7 +37719,7 @@
       </c>
       <c r="HB52" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC52" t="inlineStr">
@@ -37732,7 +37732,7 @@
       </c>
       <c r="HE52" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -38426,7 +38426,7 @@
       </c>
       <c r="HB53" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC53" t="inlineStr">
@@ -38439,7 +38439,7 @@
       </c>
       <c r="HE53" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -39137,7 +39137,7 @@
       </c>
       <c r="HB54" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC54" t="inlineStr">
@@ -39150,7 +39150,7 @@
       </c>
       <c r="HE54" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -39848,7 +39848,7 @@
       </c>
       <c r="HB55" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC55" t="inlineStr">
@@ -39861,7 +39861,7 @@
       </c>
       <c r="HE55" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -40559,7 +40559,7 @@
       </c>
       <c r="HB56" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC56" t="inlineStr">
@@ -40572,7 +40572,7 @@
       </c>
       <c r="HE56" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -41270,7 +41270,7 @@
       </c>
       <c r="HB57" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC57" t="inlineStr">
@@ -41283,7 +41283,7 @@
       </c>
       <c r="HE57" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -41981,7 +41981,7 @@
       </c>
       <c r="HB58" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC58" t="inlineStr">
@@ -41994,7 +41994,7 @@
       </c>
       <c r="HE58" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -42692,7 +42692,7 @@
       </c>
       <c r="HB59" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC59" t="inlineStr">
@@ -42705,7 +42705,7 @@
       </c>
       <c r="HE59" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -43403,7 +43403,7 @@
       </c>
       <c r="HB60" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC60" t="inlineStr">
@@ -43416,7 +43416,7 @@
       </c>
       <c r="HE60" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -44114,7 +44114,7 @@
       </c>
       <c r="HB61" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC61" t="inlineStr">
@@ -44127,7 +44127,7 @@
       </c>
       <c r="HE61" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -44825,7 +44825,7 @@
       </c>
       <c r="HB62" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC62" t="inlineStr">
@@ -44838,7 +44838,7 @@
       </c>
       <c r="HE62" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -45536,7 +45536,7 @@
       </c>
       <c r="HB63" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC63" t="inlineStr">
@@ -45549,7 +45549,7 @@
       </c>
       <c r="HE63" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -46243,7 +46243,7 @@
       </c>
       <c r="HB64" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC64" t="inlineStr">
@@ -46256,7 +46256,7 @@
       </c>
       <c r="HE64" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -46954,7 +46954,7 @@
       </c>
       <c r="HB65" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC65" t="inlineStr">
@@ -46967,7 +46967,7 @@
       </c>
       <c r="HE65" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -47665,7 +47665,7 @@
       </c>
       <c r="HB66" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC66" t="inlineStr">
@@ -47678,7 +47678,7 @@
       </c>
       <c r="HE66" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -48372,7 +48372,7 @@
       </c>
       <c r="HB67" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC67" t="inlineStr">
@@ -48385,7 +48385,7 @@
       </c>
       <c r="HE67" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -49079,7 +49079,7 @@
       </c>
       <c r="HB68" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC68" t="inlineStr">
@@ -49092,7 +49092,7 @@
       </c>
       <c r="HE68" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -49786,7 +49786,7 @@
       </c>
       <c r="HB69" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC69" t="inlineStr">
@@ -49799,7 +49799,7 @@
       </c>
       <c r="HE69" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -50497,7 +50497,7 @@
       </c>
       <c r="HB70" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC70" t="inlineStr">
@@ -50510,7 +50510,7 @@
       </c>
       <c r="HE70" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -51208,7 +51208,7 @@
       </c>
       <c r="HB71" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC71" t="inlineStr">
@@ -51221,7 +51221,7 @@
       </c>
       <c r="HE71" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -51919,7 +51919,7 @@
       </c>
       <c r="HB72" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC72" t="inlineStr">
@@ -51932,7 +51932,7 @@
       </c>
       <c r="HE72" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -52626,7 +52626,7 @@
       </c>
       <c r="HB73" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC73" t="inlineStr">
@@ -52639,7 +52639,7 @@
       </c>
       <c r="HE73" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -53337,7 +53337,7 @@
       </c>
       <c r="HB74" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC74" t="inlineStr">
@@ -53350,7 +53350,7 @@
       </c>
       <c r="HE74" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -54048,7 +54048,7 @@
       </c>
       <c r="HB75" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC75" t="inlineStr">
@@ -54061,7 +54061,7 @@
       </c>
       <c r="HE75" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -54759,7 +54759,7 @@
       </c>
       <c r="HB76" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC76" t="inlineStr">
@@ -54772,7 +54772,7 @@
       </c>
       <c r="HE76" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -55470,7 +55470,7 @@
       </c>
       <c r="HB77" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC77" t="inlineStr">
@@ -55483,7 +55483,7 @@
       </c>
       <c r="HE77" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -56177,7 +56177,7 @@
       </c>
       <c r="HB78" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC78" t="inlineStr">
@@ -56190,7 +56190,7 @@
       </c>
       <c r="HE78" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -56884,7 +56884,7 @@
       </c>
       <c r="HB79" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC79" t="inlineStr">
@@ -56897,7 +56897,7 @@
       </c>
       <c r="HE79" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -57591,7 +57591,7 @@
       </c>
       <c r="HB80" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC80" t="inlineStr">
@@ -57604,7 +57604,7 @@
       </c>
       <c r="HE80" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -58302,7 +58302,7 @@
       </c>
       <c r="HB81" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC81" t="inlineStr">
@@ -58315,7 +58315,7 @@
       </c>
       <c r="HE81" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -59009,7 +59009,7 @@
       </c>
       <c r="HB82" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC82" t="inlineStr">
@@ -59022,7 +59022,7 @@
       </c>
       <c r="HE82" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -59720,7 +59720,7 @@
       </c>
       <c r="HB83" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC83" t="inlineStr">
@@ -59733,7 +59733,7 @@
       </c>
       <c r="HE83" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -60427,7 +60427,7 @@
       </c>
       <c r="HB84" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC84" t="inlineStr">
@@ -60440,7 +60440,7 @@
       </c>
       <c r="HE84" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -61134,7 +61134,7 @@
       </c>
       <c r="HB85" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC85" t="inlineStr">
@@ -61147,7 +61147,7 @@
       </c>
       <c r="HE85" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -61841,7 +61841,7 @@
       </c>
       <c r="HB86" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC86" t="inlineStr">
@@ -61854,7 +61854,7 @@
       </c>
       <c r="HE86" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -62548,7 +62548,7 @@
       </c>
       <c r="HB87" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC87" t="inlineStr">
@@ -62561,7 +62561,7 @@
       </c>
       <c r="HE87" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -63255,7 +63255,7 @@
       </c>
       <c r="HB88" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC88" t="inlineStr">
@@ -63268,7 +63268,7 @@
       </c>
       <c r="HE88" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -63966,7 +63966,7 @@
       </c>
       <c r="HB89" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC89" t="inlineStr">
@@ -63979,7 +63979,7 @@
       </c>
       <c r="HE89" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -64673,7 +64673,7 @@
       </c>
       <c r="HB90" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC90" t="inlineStr">
@@ -64686,7 +64686,7 @@
       </c>
       <c r="HE90" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -65380,7 +65380,7 @@
       </c>
       <c r="HB91" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC91" t="inlineStr">
@@ -65393,7 +65393,7 @@
       </c>
       <c r="HE91" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -66087,7 +66087,7 @@
       </c>
       <c r="HB92" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC92" t="inlineStr">
@@ -66100,7 +66100,7 @@
       </c>
       <c r="HE92" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -66798,7 +66798,7 @@
       </c>
       <c r="HB93" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC93" t="inlineStr">
@@ -66811,7 +66811,7 @@
       </c>
       <c r="HE93" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -67509,7 +67509,7 @@
       </c>
       <c r="HB94" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC94" t="inlineStr">
@@ -67522,7 +67522,7 @@
       </c>
       <c r="HE94" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -68220,7 +68220,7 @@
       </c>
       <c r="HB95" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC95" t="inlineStr">
@@ -68233,7 +68233,7 @@
       </c>
       <c r="HE95" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -68931,7 +68931,7 @@
       </c>
       <c r="HB96" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC96" t="inlineStr">
@@ -68944,7 +68944,7 @@
       </c>
       <c r="HE96" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -69638,7 +69638,7 @@
       </c>
       <c r="HB97" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC97" t="inlineStr">
@@ -69651,7 +69651,7 @@
       </c>
       <c r="HE97" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -70349,7 +70349,7 @@
       </c>
       <c r="HB98" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC98" t="inlineStr">
@@ -70362,7 +70362,7 @@
       </c>
       <c r="HE98" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -71060,7 +71060,7 @@
       </c>
       <c r="HB99" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC99" t="inlineStr">
@@ -71073,7 +71073,7 @@
       </c>
       <c r="HE99" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -71771,7 +71771,7 @@
       </c>
       <c r="HB100" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC100" t="inlineStr">
@@ -71784,7 +71784,7 @@
       </c>
       <c r="HE100" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -72478,7 +72478,7 @@
       </c>
       <c r="HB101" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC101" t="inlineStr">
@@ -72491,7 +72491,7 @@
       </c>
       <c r="HE101" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -73185,7 +73185,7 @@
       </c>
       <c r="HB102" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC102" t="inlineStr">
@@ -73198,7 +73198,7 @@
       </c>
       <c r="HE102" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -73896,7 +73896,7 @@
       </c>
       <c r="HB103" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC103" t="inlineStr">
@@ -73909,7 +73909,7 @@
       </c>
       <c r="HE103" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -74603,7 +74603,7 @@
       </c>
       <c r="HB104" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC104" t="inlineStr">
@@ -74616,7 +74616,7 @@
       </c>
       <c r="HE104" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -75310,7 +75310,7 @@
       </c>
       <c r="HB105" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC105" t="inlineStr">
@@ -75323,7 +75323,7 @@
       </c>
       <c r="HE105" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -76017,7 +76017,7 @@
       </c>
       <c r="HB106" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC106" t="inlineStr">
@@ -76030,7 +76030,7 @@
       </c>
       <c r="HE106" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -76724,7 +76724,7 @@
       </c>
       <c r="HB107" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC107" t="inlineStr">
@@ -76737,7 +76737,7 @@
       </c>
       <c r="HE107" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -77431,7 +77431,7 @@
       </c>
       <c r="HB108" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC108" t="inlineStr">
@@ -77444,7 +77444,7 @@
       </c>
       <c r="HE108" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -78138,7 +78138,7 @@
       </c>
       <c r="HB109" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC109" t="inlineStr">
@@ -78151,7 +78151,7 @@
       </c>
       <c r="HE109" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -78845,7 +78845,7 @@
       </c>
       <c r="HB110" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC110" t="inlineStr">
@@ -78858,7 +78858,7 @@
       </c>
       <c r="HE110" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -79552,7 +79552,7 @@
       </c>
       <c r="HB111" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC111" t="inlineStr">
@@ -79565,7 +79565,7 @@
       </c>
       <c r="HE111" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -80263,7 +80263,7 @@
       </c>
       <c r="HB112" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC112" t="inlineStr">
@@ -80276,7 +80276,7 @@
       </c>
       <c r="HE112" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -80970,7 +80970,7 @@
       </c>
       <c r="HB113" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC113" t="inlineStr">
@@ -80983,7 +80983,7 @@
       </c>
       <c r="HE113" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -81677,7 +81677,7 @@
       </c>
       <c r="HB114" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC114" t="inlineStr">
@@ -81690,7 +81690,7 @@
       </c>
       <c r="HE114" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -82384,7 +82384,7 @@
       </c>
       <c r="HB115" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC115" t="inlineStr">
@@ -82397,7 +82397,7 @@
       </c>
       <c r="HE115" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -83095,7 +83095,7 @@
       </c>
       <c r="HB116" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC116" t="inlineStr">
@@ -83108,7 +83108,7 @@
       </c>
       <c r="HE116" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -83802,7 +83802,7 @@
       </c>
       <c r="HB117" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC117" t="inlineStr">
@@ -83815,7 +83815,7 @@
       </c>
       <c r="HE117" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -84509,7 +84509,7 @@
       </c>
       <c r="HB118" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC118" t="inlineStr">
@@ -84522,7 +84522,7 @@
       </c>
       <c r="HE118" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -85216,7 +85216,7 @@
       </c>
       <c r="HB119" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC119" t="inlineStr">
@@ -85229,7 +85229,7 @@
       </c>
       <c r="HE119" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -85923,7 +85923,7 @@
       </c>
       <c r="HB120" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC120" t="inlineStr">
@@ -85936,7 +85936,7 @@
       </c>
       <c r="HE120" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>
@@ -86630,7 +86630,7 @@
       </c>
       <c r="HB121" t="inlineStr">
         <is>
-          <t>2026-05-28T20:48:12.054844-04:00</t>
+          <t>2026-05-28T22:10:01.247694-04:00</t>
         </is>
       </c>
       <c r="HC121" t="inlineStr">
@@ -86643,7 +86643,7 @@
       </c>
       <c r="HE121" t="inlineStr">
         <is>
-          <t>2026-05-28 08:48:12 PM</t>
+          <t>2026-05-28 10:10:01 PM</t>
         </is>
       </c>
     </row>

</xml_diff>